<commit_message>
remove too much classifcation info
</commit_message>
<xml_diff>
--- a/excercise2/classification/LoR/LoR_top_features.xlsx
+++ b/excercise2/classification/LoR/LoR_top_features.xlsx
@@ -1,20 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\IR\IR2026\excercise2\classification\LoR\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -33,67 +28,64 @@
     <t>class_label</t>
   </si>
   <si>
-    <t>194</t>
-  </si>
-  <si>
-    <t>169</t>
+    <t>roger</t>
+  </si>
+  <si>
+    <t>williams</t>
+  </si>
+  <si>
+    <t>texas</t>
+  </si>
+  <si>
+    <t>x27</t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>december</t>
+  </si>
+  <si>
+    <t>digest</t>
+  </si>
+  <si>
+    <t>senate</t>
+  </si>
+  <si>
+    <t>computerized</t>
+  </si>
+  <si>
+    <t>computerization</t>
+  </si>
+  <si>
+    <t>extensions</t>
   </si>
   <si>
     <t>remarks</t>
   </si>
   <si>
-    <t>congressional</t>
-  </si>
-  <si>
-    <t>www</t>
-  </si>
-  <si>
-    <t>gpo</t>
-  </si>
-  <si>
-    <t>href</t>
-  </si>
-  <si>
-    <t>https</t>
-  </si>
-  <si>
-    <t>170</t>
-  </si>
-  <si>
-    <t>publishing</t>
-  </si>
-  <si>
-    <t>pages</t>
-  </si>
-  <si>
-    <t>gov</t>
-  </si>
-  <si>
-    <t>x27</t>
+    <t>subcommittee</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>rules</t>
+  </si>
+  <si>
+    <t>iv</t>
+  </si>
+  <si>
+    <t>1977</t>
+  </si>
+  <si>
+    <t>recognize</t>
   </si>
   <si>
     <t>title</t>
   </si>
   <si>
-    <t>digest</t>
-  </si>
-  <si>
-    <t>roger</t>
-  </si>
-  <si>
-    <t>senate</t>
-  </si>
-  <si>
-    <t>volume</t>
-  </si>
-  <si>
-    <t>williams</t>
-  </si>
-  <si>
-    <t>171</t>
-  </si>
-  <si>
-    <t>uk</t>
+    <t>friday</t>
   </si>
   <si>
     <t>labour</t>
@@ -129,18 +121,18 @@
     <t>programme</t>
   </si>
   <si>
+    <t>centre</t>
+  </si>
+  <si>
+    <t>minister</t>
+  </si>
+  <si>
+    <t>prime</t>
+  </si>
+  <si>
     <t>scotland</t>
   </si>
   <si>
-    <t>centre</t>
-  </si>
-  <si>
-    <t>prime</t>
-  </si>
-  <si>
-    <t>minister</t>
-  </si>
-  <si>
     <t>debate</t>
   </si>
   <si>
@@ -148,6 +140,9 @@
   </si>
   <si>
     <t>shadow</t>
+  </si>
+  <si>
+    <t>maiden</t>
   </si>
   <si>
     <t>discuss</t>
@@ -162,12 +157,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -175,7 +170,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -226,19 +221,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -280,7 +267,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -312,10 +299,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -347,7 +333,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -523,17 +508,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,561 +526,561 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.13719262792538539</v>
+        <v>0.2087686806103504</v>
       </c>
       <c r="C2">
-        <v>0.13719262792538539</v>
+        <v>0.2087686806103504</v>
       </c>
       <c r="D2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0.1091073281809907</v>
+        <v>0.1766863004579825</v>
       </c>
       <c r="C3">
-        <v>0.1091073281809907</v>
+        <v>0.1766863004579825</v>
       </c>
       <c r="D3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.10638663088232431</v>
+        <v>0.129304384259268</v>
       </c>
       <c r="C4">
-        <v>0.10638663088232431</v>
+        <v>0.129304384259268</v>
       </c>
       <c r="D4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5">
-        <v>0.1062093763442282</v>
+        <v>0.1122135432846981</v>
       </c>
       <c r="C5">
-        <v>0.1062093763442282</v>
+        <v>0.1122135432846981</v>
       </c>
       <c r="D5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0.1047722465024971</v>
+        <v>0.110778745047303</v>
       </c>
       <c r="C6">
-        <v>0.1047722465024971</v>
+        <v>0.110778745047303</v>
       </c>
       <c r="D6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7">
-        <v>0.10477194104888291</v>
+        <v>0.09978486044011078</v>
       </c>
       <c r="C7">
-        <v>0.10477194104888291</v>
+        <v>0.09978486044011078</v>
       </c>
       <c r="D7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8">
-        <v>9.2952905962903218E-2</v>
+        <v>0.09914557570814202</v>
       </c>
       <c r="C8">
-        <v>9.2952905962903218E-2</v>
+        <v>0.09914557570814202</v>
       </c>
       <c r="D8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>11</v>
       </c>
       <c r="B9">
-        <v>9.2952843555330719E-2</v>
+        <v>0.08938379604446389</v>
       </c>
       <c r="C9">
-        <v>9.2952843555330719E-2</v>
+        <v>0.08938379604446389</v>
       </c>
       <c r="D9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>12</v>
       </c>
       <c r="B10">
-        <v>9.209999257840977E-2</v>
+        <v>0.0838868751602955</v>
       </c>
       <c r="C10">
-        <v>9.209999257840977E-2</v>
+        <v>0.0838868751602955</v>
       </c>
       <c r="D10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11">
-        <v>8.9200612238600305E-2</v>
+        <v>0.0838868751602955</v>
       </c>
       <c r="C11">
-        <v>8.9200612238600305E-2</v>
+        <v>0.0838868751602955</v>
       </c>
       <c r="D11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>14</v>
       </c>
       <c r="B12">
-        <v>8.5770017563065917E-2</v>
+        <v>0.08388202731778847</v>
       </c>
       <c r="C12">
-        <v>8.5770017563065917E-2</v>
+        <v>0.08388202731778847</v>
       </c>
       <c r="D12" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>15</v>
       </c>
       <c r="B13">
-        <v>8.4356110702740683E-2</v>
+        <v>0.08311893403677509</v>
       </c>
       <c r="C13">
-        <v>8.4356110702740683E-2</v>
+        <v>0.08311893403677509</v>
       </c>
       <c r="D13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14">
-        <v>8.276465145827569E-2</v>
+        <v>0.0813511470551283</v>
       </c>
       <c r="C14">
-        <v>8.276465145827569E-2</v>
+        <v>0.0813511470551283</v>
       </c>
       <c r="D14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>17</v>
       </c>
       <c r="B15">
-        <v>7.8582214094855787E-2</v>
+        <v>0.0805780725588988</v>
       </c>
       <c r="C15">
-        <v>7.8582214094855787E-2</v>
+        <v>0.0805780725588988</v>
       </c>
       <c r="D15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>18</v>
       </c>
       <c r="B16">
-        <v>7.322422102773686E-2</v>
+        <v>0.07935619036806681</v>
       </c>
       <c r="C16">
-        <v>7.322422102773686E-2</v>
+        <v>0.07935619036806681</v>
       </c>
       <c r="D16" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>19</v>
       </c>
       <c r="B17">
-        <v>7.1052456147740986E-2</v>
+        <v>0.07482853922694374</v>
       </c>
       <c r="C17">
-        <v>7.1052456147740986E-2</v>
+        <v>0.07482853922694374</v>
       </c>
       <c r="D17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
       <c r="B18">
-        <v>6.8440697861170782E-2</v>
+        <v>0.07327048263532977</v>
       </c>
       <c r="C18">
-        <v>6.8440697861170782E-2</v>
+        <v>0.07327048263532977</v>
       </c>
       <c r="D18" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>21</v>
       </c>
       <c r="B19">
-        <v>6.5418077218746915E-2</v>
+        <v>0.07024628226508448</v>
       </c>
       <c r="C19">
-        <v>6.5418077218746915E-2</v>
+        <v>0.07024628226508448</v>
       </c>
       <c r="D19" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>22</v>
       </c>
       <c r="B20">
-        <v>6.4172846083684357E-2</v>
+        <v>0.0694621461071513</v>
       </c>
       <c r="C20">
-        <v>6.4172846083684357E-2</v>
+        <v>0.0694621461071513</v>
       </c>
       <c r="D20" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
       <c r="B21">
-        <v>6.2648728048838809E-2</v>
+        <v>0.06910164795332541</v>
       </c>
       <c r="C21">
-        <v>6.2648728048838809E-2</v>
+        <v>0.06910164795332541</v>
       </c>
       <c r="D21" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>24</v>
       </c>
       <c r="B22">
-        <v>-2.4143445141133851E-2</v>
+        <v>-0.02573077902375551</v>
       </c>
       <c r="C22">
-        <v>2.4143445141133851E-2</v>
+        <v>0.02573077902375551</v>
       </c>
       <c r="D22" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>25</v>
       </c>
       <c r="B23">
-        <v>-2.3332942337918661E-2</v>
+        <v>-0.02538219370269464</v>
       </c>
       <c r="C23">
-        <v>2.3332942337918661E-2</v>
+        <v>0.02538219370269464</v>
       </c>
       <c r="D23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>26</v>
       </c>
       <c r="B24">
-        <v>-2.3003698154185379E-2</v>
+        <v>-0.02317042763572257</v>
       </c>
       <c r="C24">
-        <v>2.3003698154185379E-2</v>
+        <v>0.02317042763572257</v>
       </c>
       <c r="D24" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>27</v>
       </c>
       <c r="B25">
-        <v>-2.11026897699816E-2</v>
+        <v>-0.02281805772677934</v>
       </c>
       <c r="C25">
-        <v>2.11026897699816E-2</v>
+        <v>0.02281805772677934</v>
       </c>
       <c r="D25" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>28</v>
       </c>
       <c r="B26">
-        <v>-2.062207052409366E-2</v>
+        <v>-0.02128532615003247</v>
       </c>
       <c r="C26">
-        <v>2.062207052409366E-2</v>
+        <v>0.02128532615003247</v>
       </c>
       <c r="D26" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>29</v>
       </c>
       <c r="B27">
-        <v>-1.9481648566600659E-2</v>
+        <v>-0.0212811880289111</v>
       </c>
       <c r="C27">
-        <v>1.9481648566600659E-2</v>
+        <v>0.0212811880289111</v>
       </c>
       <c r="D27" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>30</v>
       </c>
       <c r="B28">
-        <v>-1.922108623302423E-2</v>
+        <v>-0.02079525062392902</v>
       </c>
       <c r="C28">
-        <v>1.922108623302423E-2</v>
+        <v>0.02079525062392902</v>
       </c>
       <c r="D28" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>31</v>
       </c>
       <c r="B29">
-        <v>-1.892069808818081E-2</v>
+        <v>-0.02048058738670841</v>
       </c>
       <c r="C29">
-        <v>1.892069808818081E-2</v>
+        <v>0.02048058738670841</v>
       </c>
       <c r="D29" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>32</v>
       </c>
       <c r="B30">
-        <v>-1.8655401870116911E-2</v>
+        <v>-0.02023967044928879</v>
       </c>
       <c r="C30">
-        <v>1.8655401870116911E-2</v>
+        <v>0.02023967044928879</v>
       </c>
       <c r="D30" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>33</v>
       </c>
       <c r="B31">
-        <v>-1.8292105365467621E-2</v>
+        <v>-0.02004203841151398</v>
       </c>
       <c r="C31">
-        <v>1.8292105365467621E-2</v>
+        <v>0.02004203841151398</v>
       </c>
       <c r="D31" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4">
       <c r="A32" t="s">
         <v>34</v>
       </c>
       <c r="B32">
-        <v>-1.822533250687336E-2</v>
+        <v>-0.01951485890265312</v>
       </c>
       <c r="C32">
-        <v>1.822533250687336E-2</v>
+        <v>0.01951485890265312</v>
       </c>
       <c r="D32" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4">
       <c r="A33" t="s">
         <v>35</v>
       </c>
       <c r="B33">
-        <v>-1.7892331899398369E-2</v>
+        <v>-0.01950552166636415</v>
       </c>
       <c r="C33">
-        <v>1.7892331899398369E-2</v>
+        <v>0.01950552166636415</v>
       </c>
       <c r="D33" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4">
       <c r="A34" t="s">
         <v>36</v>
       </c>
       <c r="B34">
-        <v>-1.7725301281980788E-2</v>
+        <v>-0.01949327941384968</v>
       </c>
       <c r="C34">
-        <v>1.7725301281980788E-2</v>
+        <v>0.01949327941384968</v>
       </c>
       <c r="D34" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4">
       <c r="A35" t="s">
         <v>37</v>
       </c>
       <c r="B35">
-        <v>-1.7573963953757661E-2</v>
+        <v>-0.01933962269764145</v>
       </c>
       <c r="C35">
-        <v>1.7573963953757661E-2</v>
+        <v>0.01933962269764145</v>
       </c>
       <c r="D35" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4">
       <c r="A36" t="s">
         <v>38</v>
       </c>
       <c r="B36">
-        <v>-1.7407419228407311E-2</v>
+        <v>-0.01926887310089744</v>
       </c>
       <c r="C36">
-        <v>1.7407419228407311E-2</v>
+        <v>0.01926887310089744</v>
       </c>
       <c r="D36" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>39</v>
       </c>
       <c r="B37">
-        <v>-1.7390600590103968E-2</v>
+        <v>-0.01917650971619386</v>
       </c>
       <c r="C37">
-        <v>1.7390600590103968E-2</v>
+        <v>0.01917650971619386</v>
       </c>
       <c r="D37" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4">
       <c r="A38" t="s">
         <v>40</v>
       </c>
       <c r="B38">
-        <v>-1.7238781383214111E-2</v>
+        <v>-0.01893717781736507</v>
       </c>
       <c r="C38">
-        <v>1.7238781383214111E-2</v>
+        <v>0.01893717781736507</v>
       </c>
       <c r="D38" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4">
       <c r="A39" t="s">
         <v>41</v>
       </c>
       <c r="B39">
-        <v>-1.723590356686152E-2</v>
+        <v>-0.01889852928595741</v>
       </c>
       <c r="C39">
-        <v>1.723590356686152E-2</v>
+        <v>0.01889852928595741</v>
       </c>
       <c r="D39" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>42</v>
       </c>
       <c r="B40">
-        <v>-1.7209319270823819E-2</v>
+        <v>-0.01870415292384537</v>
       </c>
       <c r="C40">
-        <v>1.7209319270823819E-2</v>
+        <v>0.01870415292384537</v>
       </c>
       <c r="D40" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
         <v>43</v>
       </c>
       <c r="B41">
-        <v>-1.7140274640651331E-2</v>
+        <v>-0.01867227488292616</v>
       </c>
       <c r="C41">
-        <v>1.7140274640651331E-2</v>
+        <v>0.01867227488292616</v>
       </c>
       <c r="D41" t="s">
         <v>45</v>

</xml_diff>